<commit_message>
[P2] add preview snapshot, fix balance.xlsx, add workflow rules to AI_CONTEXT
- Add 功夫足球_preview.html to git tracking (remove from .gitignore)

- Add dribbleBaseSuccess/interceptBaseChance/blockBaseChance to balance.xlsx

- Regenerate balance.json with 10 entries

- Add Section 11 workflow rules to AI_CONTEXT.md for agent visibility

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/data/balance.xlsx
+++ b/data/balance.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -511,9 +511,51 @@
         <v>传球后射门概率</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>dribbleBaseSuccess</v>
+      </c>
+      <c r="B9">
+        <v>0.55</v>
+      </c>
+      <c r="C9" t="str">
+        <v>number</v>
+      </c>
+      <c r="D9" t="str">
+        <v>带球过人基础成功率</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>interceptBaseChance</v>
+      </c>
+      <c r="B10">
+        <v>0.4</v>
+      </c>
+      <c r="C10" t="str">
+        <v>number</v>
+      </c>
+      <c r="D10" t="str">
+        <v>防守方尝试拦截传球的概率</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>blockBaseChance</v>
+      </c>
+      <c r="B11">
+        <v>0.25</v>
+      </c>
+      <c r="C11" t="str">
+        <v>number</v>
+      </c>
+      <c r="D11" t="str">
+        <v>防守方尝试封堵射门的概率</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>